<commit_message>
feat: schema v1.0/v1.1 版本化 + 迁移机制 + Excel 计算模板模糊化
- Schema 版本化：v1.0 历史快照（不可变）+ v1.1 新增 3 个可选字段
  - valuation.estimatedDate（预计成交日期）
  - result.calculationMode（结果确定方式 enum）
  - crossMethodNotes（跨方法综合讨论笔记）
- 迁移脚本 migrate_schema.py：1.0→1.1 自动补全 + 预览模式 + 同版本 skip
- 验证器更新：detect_version + validate_full 版本路由
- Excel 评估明细表模糊化 → 计算模板（11 sheet, 1582 公式完整保留）
- 模糊化脚本 anonymize_template.py：通用化重构，命令行参数传入源文件
- CHANGELOG.md：Semantic Versioning 变更日志
- 交接文档 HANDOFF-2026-08-13.md：自包含，不依赖对话上下文
- 测试：117/117 全绿（新增 29 个版本化迁移测试）
- 安全：全仓库敏感信息扫描通过，真实姓名/地址/楼盘名/网络路径已清除
</commit_message>
<xml_diff>
--- a/outputs/templates/假设开发法测算_模板.xlsx
+++ b/outputs/templates/假设开发法测算_模板.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="假设开发法" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="现金流时间线" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="假设开发法" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="现金流时间线" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
feat(schema): v1.3 人工决策点 decisionPoints
新增 decisionPoints 可选字段 + 4 个 （decisionPoint/evidenceItem/riskItem/comparisonItem），
支持 AI 在关键专业判断节点暂停等待估价师批准/调整/驳回。

变更：
- schema/appraisal-result.schema.json: schemaVersion ^1.2$ → ^1.3$，新增 decisionPoints 属性
- schema/v1.3/: 版本化副本
- schema/example-武汉洪山住宅.json: 升级到 v1.3，填充 6 个决策点示例（DP1-DP4 + DP-comp + DP-income）
- scripts/validate_appraisal_json.py: VERSION_SCHEMA_MAP 加 1.3
- scripts/migrate_schema.py: 新增 _migrate_1_2_to_1_3() 迁移路径
- tests/test_schema_v13.py: 44 个测试（7 类）
- tests/: 修复 v1.3 升级导致的 15 个回归（_strip_v12_fields 剥离 decisionPoints、
  v1.2 测试用 _strip_v13_fields 创建 v1.2 base、degradation fixture 升级到 1.3）
- CHANGELOG.md: v1.3 条目

全量测试 230/230 通过。
</commit_message>
<xml_diff>
--- a/outputs/templates/假设开发法测算_模板.xlsx
+++ b/outputs/templates/假设开发法测算_模板.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="假设开发法" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="现金流时间线" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="假设开发法" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="现金流时间线" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
fix(scripts): preserve inline xmlns declarations when freezing core.xml
save_frozen() replaced the whole created/modified tag with a hardcoded
string, swallowing the inline xmlns:dcterms / xmlns:xsi declarations that
openpyxl 3.1.5 now emits on the element itself (not the root). The result
was malformed core.xml and XMLSyntaxError on read-back (28 test_templates
failures). Replace only the timestamp text and keep the opening tag
verbatim; regenerate all 4 templates.
</commit_message>
<xml_diff>
--- a/outputs/templates/假设开发法测算_模板.xlsx
+++ b/outputs/templates/假设开发法测算_模板.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="假设开发法" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="现金流时间线" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="假设开发法" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="现金流时间线" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>